<commit_message>
revert(ornek): ornek-tedarik-listesi.xlsx d287c3e oncesi haline dondu
Excel dosyayi acikken yeniden kaydetmis, d287c3e'de 'git add -A' ile istem disi
suruklendi (13.900 -> 34.283 bayt). Icerik degisikligi amaclanmadi; PM onayiyla
revert. Not: dosya lokalde Excel tarafindan kilitli oldugu icin calisma
kopyasi guncellenmedi; depodaki hali dogru.
</commit_message>
<xml_diff>
--- a/ornek-tedarik-listesi.xlsx
+++ b/ornek-tedarik-listesi.xlsx
@@ -3,12 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\tedarikapp\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2E19B665-A189-4799-8BFA-5DA009EDDFC9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92A3A747-F5F6-41FF-83D0-7CCD064E95E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,9 +23,15 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="25">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="17">
+  <si>
+    <t>ÜRÜN GÖRSELİ</t>
+  </si>
   <si>
     <t>ÜRÜN ADI</t>
+  </si>
+  <si>
+    <t>1688 FİYATI</t>
   </si>
   <si>
     <t>DDP FİYATI</t>
@@ -71,53 +72,22 @@
     <t>KATEGORİ</t>
   </si>
   <si>
+    <t>ÜRÜN DETAY</t>
+  </si>
+  <si>
+    <t>ÜRÜN LİNKİ</t>
+  </si>
+  <si>
+    <t>https://detail.1688.com/offer/000000000000.html</t>
+  </si>
+  <si>
     <t>MUTFAK</t>
   </si>
   <si>
     <t>Örnek detay: 500 ml · paslanmaz çelik · gri</t>
   </si>
   <si>
-    <t>Örnek Ürün — Termos Yemek Kabı</t>
-  </si>
-  <si>
-    <t>ELEKTRONİK</t>
-  </si>
-  <si>
-    <t>DEKORASYON</t>
-  </si>
-  <si>
-    <t>KAYNAK</t>
-  </si>
-  <si>
-    <t>ÇİN PARAKENDE</t>
-  </si>
-  <si>
-    <t>DURUM</t>
-  </si>
-  <si>
-    <t>İPTAL EDİLDİ</t>
-  </si>
-  <si>
-    <t>SİPARİŞ VERİLDİ</t>
-  </si>
-  <si>
-    <t>BEKLEMEDE</t>
-  </si>
-  <si>
-    <t>GÖRSEL</t>
-  </si>
-  <si>
-    <t>NOT</t>
-  </si>
-  <si>
-    <t>ÜRÜN DETAYLARI</t>
-  </si>
-  <si>
-    <t>,</t>
-  </si>
-  <si>
-    <t>ürün kutusu 
-logolu olacak</t>
+    <t xml:space="preserve">Örnek Ürün — Termos Yemek Kabı</t>
   </si>
 </sst>
 </file>
@@ -129,7 +99,7 @@
     <numFmt numFmtId="165" formatCode="&quot;₺&quot;#,##0.00"/>
     <numFmt numFmtId="166" formatCode="[$$-409]#,##0.00"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -144,6 +114,14 @@
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="162"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -188,46 +166,8 @@
       <charset val="162"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF006100"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="162"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C0006"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="162"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color rgb="FF9C5700"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="162"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="14"/>
-      <color theme="1"/>
-      <name val="Calibri Light"/>
-      <family val="2"/>
-      <charset val="162"/>
-      <scheme val="major"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Arial Tur"/>
-      <charset val="162"/>
-    </font>
   </fonts>
-  <fills count="9">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -258,23 +198,8 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFC6EFCE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFC7CE"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFEB9C"/>
-      </patternFill>
-    </fill>
   </fills>
-  <borders count="8">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -357,131 +282,77 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="FF3F3F3F"/>
-      </left>
-      <right style="thin">
-        <color rgb="FF3F3F3F"/>
-      </right>
-      <top style="thin">
-        <color rgb="FF3F3F3F"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="FF3F3F3F"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="medium">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
-  <cellStyleXfs count="4">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="4" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="4" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="5" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="6" borderId="6" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="1" xfId="2" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="1" xfId="3" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="4">
-    <cellStyle name="İyi" xfId="1" builtinId="26"/>
-    <cellStyle name="Kötü" xfId="2" builtinId="27"/>
+  <cellStyles count="2">
+    <cellStyle name="Köprü" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Nötr" xfId="3" builtinId="28"/>
   </cellStyles>
   <dxfs count="1">
     <dxf>
@@ -512,13 +383,13 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>66675</xdr:colOff>
+      <xdr:colOff>428625</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>47625</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1276350</xdr:colOff>
+      <xdr:colOff>1638300</xdr:colOff>
       <xdr:row>8</xdr:row>
       <xdr:rowOff>981075</xdr:rowOff>
     </xdr:to>
@@ -549,158 +420,7 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="1057275" y="1628775"/>
-          <a:ext cx="1209675" cy="933450"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>142875</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>133350</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>857250</xdr:colOff>
-      <xdr:row>8</xdr:row>
-      <xdr:rowOff>847725</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Resim 3">
-          <a:hlinkClick xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A8ACAC88-9241-45C9-AF9E-D7FFC6501F31}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId3" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="8648700" y="1714500"/>
-          <a:ext cx="714375" cy="714375"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>66675</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>38100</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1276350</xdr:colOff>
-      <xdr:row>9</xdr:row>
-      <xdr:rowOff>971550</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="5" name="Resim 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5783C590-5EF6-43D0-AF00-46A66C8F4186}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="962025" y="2628900"/>
-          <a:ext cx="1209675" cy="933450"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>66675</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>1276350</xdr:colOff>
-      <xdr:row>10</xdr:row>
-      <xdr:rowOff>981075</xdr:rowOff>
-    </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="6" name="Resim 5">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{01F99473-AD81-4C07-9D9E-598845CD02E2}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="962025" y="3648075"/>
+          <a:off x="1419225" y="1628775"/>
           <a:ext cx="1209675" cy="933450"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
@@ -976,317 +696,266 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="B2:Z504"/>
+  <dimension ref="B2:V504"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="2.85546875" style="2" customWidth="1"/>
-    <col min="2" max="2" width="9.85546875" style="2" customWidth="1"/>
+    <col min="2" max="2" width="11.28515625" style="2" customWidth="1"/>
     <col min="3" max="3" width="0.7109375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="20" style="2" customWidth="1"/>
+    <col min="4" max="4" width="34.42578125" style="2" customWidth="1"/>
     <col min="5" max="5" width="0.7109375" style="2" customWidth="1"/>
-    <col min="6" max="6" width="18.85546875" style="21" customWidth="1"/>
+    <col min="6" max="6" width="18.85546875" style="2" customWidth="1"/>
     <col min="7" max="7" width="0.7109375" style="2" customWidth="1"/>
     <col min="8" max="8" width="30.85546875" style="2" customWidth="1"/>
     <col min="9" max="9" width="0.7109375" style="2" customWidth="1"/>
     <col min="10" max="10" width="41" style="2" customWidth="1"/>
     <col min="11" max="11" width="0.7109375" style="2" customWidth="1"/>
-    <col min="12" max="12" width="14.85546875" style="2" customWidth="1"/>
+    <col min="12" max="12" width="23.85546875" style="2" customWidth="1"/>
     <col min="13" max="13" width="0.7109375" style="2" customWidth="1"/>
-    <col min="14" max="14" width="23.85546875" style="2" customWidth="1"/>
+    <col min="14" max="14" width="22.7109375" style="2" customWidth="1"/>
     <col min="15" max="15" width="0.7109375" style="2" customWidth="1"/>
-    <col min="16" max="16" width="15.28515625" style="2" customWidth="1"/>
+    <col min="16" max="16" width="12.28515625" style="2" customWidth="1"/>
     <col min="17" max="17" width="0.7109375" style="2" customWidth="1"/>
-    <col min="18" max="18" width="15.5703125" style="2" customWidth="1"/>
+    <col min="18" max="18" width="12.28515625" style="2" customWidth="1"/>
     <col min="19" max="19" width="0.7109375" style="2" customWidth="1"/>
     <col min="20" max="20" width="12.28515625" style="2" customWidth="1"/>
     <col min="21" max="21" width="0.7109375" style="2" customWidth="1"/>
     <col min="22" max="22" width="12.28515625" style="2" customWidth="1"/>
-    <col min="23" max="23" width="0.7109375" style="2" customWidth="1"/>
-    <col min="24" max="24" width="12.28515625" style="2" customWidth="1"/>
-    <col min="25" max="25" width="0.7109375" style="2" customWidth="1"/>
-    <col min="26" max="26" width="12.28515625" style="2" customWidth="1"/>
-    <col min="27" max="16384" width="9.140625" style="2"/>
+    <col min="23" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B2" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19"/>
-      <c r="G2" s="19"/>
-      <c r="H2" s="19"/>
-      <c r="I2" s="19"/>
-      <c r="J2" s="19"/>
-      <c r="K2" s="19"/>
-      <c r="L2" s="19"/>
-      <c r="M2" s="19"/>
-      <c r="N2" s="19"/>
-      <c r="O2" s="19"/>
-      <c r="P2" s="19"/>
-      <c r="Q2" s="19"/>
-      <c r="R2" s="19"/>
-      <c r="S2" s="19"/>
-      <c r="T2" s="19"/>
-      <c r="U2" s="19"/>
-      <c r="V2" s="19"/>
-      <c r="W2" s="19"/>
-      <c r="X2" s="19"/>
-      <c r="Y2" s="19"/>
-      <c r="Z2" s="19"/>
+    <row r="2" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B2" s="15" t="s">
+        <v>9</v>
+      </c>
+      <c r="C2" s="15"/>
+      <c r="D2" s="15"/>
+      <c r="E2" s="15"/>
+      <c r="F2" s="15"/>
+      <c r="G2" s="15"/>
+      <c r="H2" s="15"/>
+      <c r="I2" s="15"/>
+      <c r="J2" s="15"/>
+      <c r="K2" s="15"/>
+      <c r="L2" s="15"/>
+      <c r="M2" s="15"/>
+      <c r="N2" s="15"/>
+      <c r="O2" s="15"/>
+      <c r="P2" s="15"/>
+      <c r="Q2" s="15"/>
+      <c r="R2" s="15"/>
+      <c r="S2" s="15"/>
+      <c r="T2" s="15"/>
+      <c r="U2" s="15"/>
+      <c r="V2" s="15"/>
     </row>
-    <row r="3" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B3" s="19"/>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
-      <c r="E3" s="19"/>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
-      <c r="H3" s="19"/>
-      <c r="I3" s="19"/>
-      <c r="J3" s="19"/>
-      <c r="K3" s="19"/>
-      <c r="L3" s="19"/>
-      <c r="M3" s="19"/>
-      <c r="N3" s="19"/>
-      <c r="O3" s="19"/>
-      <c r="P3" s="19"/>
-      <c r="Q3" s="19"/>
-      <c r="R3" s="19"/>
-      <c r="S3" s="19"/>
-      <c r="T3" s="19"/>
-      <c r="U3" s="19"/>
-      <c r="V3" s="19"/>
-      <c r="W3" s="19"/>
-      <c r="X3" s="19"/>
-      <c r="Y3" s="19"/>
-      <c r="Z3" s="19"/>
+    <row r="3" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="15"/>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="15"/>
+      <c r="N3" s="15"/>
+      <c r="O3" s="15"/>
+      <c r="P3" s="15"/>
+      <c r="Q3" s="15"/>
+      <c r="R3" s="15"/>
+      <c r="S3" s="15"/>
+      <c r="T3" s="15"/>
+      <c r="U3" s="15"/>
+      <c r="V3" s="15"/>
     </row>
-    <row r="4" spans="2:26" x14ac:dyDescent="0.25">
-      <c r="B4" s="19"/>
-      <c r="C4" s="19"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="19"/>
-      <c r="F4" s="19"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="19"/>
-      <c r="I4" s="19"/>
-      <c r="J4" s="19"/>
-      <c r="K4" s="19"/>
-      <c r="L4" s="19"/>
-      <c r="M4" s="19"/>
-      <c r="N4" s="19"/>
-      <c r="O4" s="19"/>
-      <c r="P4" s="19"/>
-      <c r="Q4" s="19"/>
-      <c r="R4" s="19"/>
-      <c r="S4" s="19"/>
-      <c r="T4" s="19"/>
-      <c r="U4" s="19"/>
-      <c r="V4" s="19"/>
-      <c r="W4" s="19"/>
-      <c r="X4" s="19"/>
-      <c r="Y4" s="19"/>
-      <c r="Z4" s="19"/>
+    <row r="4" spans="2:22" x14ac:dyDescent="0.25">
+      <c r="B4" s="15"/>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="15"/>
+      <c r="H4" s="15"/>
+      <c r="I4" s="15"/>
+      <c r="J4" s="15"/>
+      <c r="K4" s="15"/>
+      <c r="L4" s="15"/>
+      <c r="M4" s="15"/>
+      <c r="N4" s="15"/>
+      <c r="O4" s="15"/>
+      <c r="P4" s="15"/>
+      <c r="Q4" s="15"/>
+      <c r="R4" s="15"/>
+      <c r="S4" s="15"/>
+      <c r="T4" s="15"/>
+      <c r="U4" s="15"/>
+      <c r="V4" s="15"/>
     </row>
-    <row r="5" spans="2:26" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:22" ht="11.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B5" s="1"/>
       <c r="C5" s="1"/>
     </row>
-    <row r="6" spans="2:26" s="1" customFormat="1" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B6" s="8" t="s">
+    <row r="6" spans="2:22" s="1" customFormat="1" ht="33" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="11" t="s">
+        <v>4</v>
+      </c>
+      <c r="D6" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="F6" s="11" t="s">
+        <v>10</v>
+      </c>
+      <c r="H6" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="J6" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="L6" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="N6" s="11" t="s">
+        <v>8</v>
+      </c>
+      <c r="P6" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="D6" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="F6" s="22" t="s">
-        <v>8</v>
-      </c>
-      <c r="H6" s="8" t="s">
-        <v>0</v>
-      </c>
-      <c r="J6" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="L6" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="N6" s="8" t="s">
-        <v>16</v>
-      </c>
-      <c r="P6" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="R6" s="20" t="s">
+      <c r="Q6" s="9"/>
+      <c r="R6" s="10"/>
+      <c r="T6" s="8" t="s">
+        <v>3</v>
+      </c>
+      <c r="U6" s="9"/>
+      <c r="V6" s="10"/>
+    </row>
+    <row r="7" spans="2:22" s="1" customFormat="1" ht="5.25" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="8" spans="2:22" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="P8" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="Q8" s="4"/>
+      <c r="R8" s="3" t="s">
         <v>6</v>
       </c>
-      <c r="T6" s="16" t="s">
-        <v>15</v>
-      </c>
-      <c r="U6" s="17"/>
-      <c r="V6" s="18"/>
-      <c r="X6" s="16" t="s">
-        <v>1</v>
-      </c>
-      <c r="Y6" s="17"/>
-      <c r="Z6" s="18"/>
-    </row>
-    <row r="7" spans="2:26" s="1" customFormat="1" ht="5.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F7" s="23"/>
-    </row>
-    <row r="8" spans="2:26" s="1" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="F8" s="23"/>
+      <c r="S8" s="4"/>
       <c r="T8" s="3" t="s">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="U8" s="4"/>
       <c r="V8" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="W8" s="4"/>
-      <c r="X8" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="Y8" s="4"/>
-      <c r="Z8" s="3" t="s">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
-    <row r="9" spans="2:26" ht="79.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:22" ht="79.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B9" s="6">
         <v>1</v>
       </c>
       <c r="C9" s="7"/>
-      <c r="D9" s="9"/>
-      <c r="E9" s="10"/>
-      <c r="F9" s="24" t="s">
-        <v>9</v>
-      </c>
-      <c r="G9" s="10"/>
-      <c r="H9" s="28" t="s">
-        <v>11</v>
-      </c>
-      <c r="I9" s="10"/>
-      <c r="J9" s="28" t="s">
-        <v>10</v>
-      </c>
-      <c r="K9" s="10"/>
-      <c r="L9" s="5"/>
-      <c r="M9" s="10"/>
-      <c r="N9" s="25" t="s">
-        <v>18</v>
-      </c>
-      <c r="O9" s="10"/>
-      <c r="P9" s="29" t="s">
+      <c r="D9" s="12"/>
+      <c r="E9" s="13"/>
+      <c r="F9" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G9" s="13"/>
+      <c r="H9" s="19" t="s">
+        <v>16</v>
+      </c>
+      <c r="I9" s="13"/>
+      <c r="J9" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="K9" s="13"/>
+      <c r="L9" s="17" t="s">
+        <v>13</v>
+      </c>
+      <c r="M9" s="13"/>
+      <c r="N9" s="5">
         <v>24</v>
       </c>
-      <c r="Q9" s="10"/>
-      <c r="R9" s="5">
-        <v>24</v>
-      </c>
-      <c r="S9" s="10"/>
-      <c r="T9" s="12">
+      <c r="O9" s="13"/>
+      <c r="P9" s="18">
         <v>12</v>
       </c>
-      <c r="U9" s="14"/>
-      <c r="V9" s="13">
+      <c r="Q9" s="21"/>
+      <c r="R9" s="20">
         <v>84.48</v>
       </c>
-      <c r="W9" s="14"/>
-      <c r="X9" s="15">
+      <c r="S9" s="21"/>
+      <c r="T9" s="22">
         <v>0</v>
       </c>
-      <c r="Y9" s="14"/>
-      <c r="Z9" s="13">
+      <c r="U9" s="21"/>
+      <c r="V9" s="20">
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="2:26" ht="79.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:22" ht="79.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B10" s="6">
         <v>2</v>
       </c>
       <c r="C10" s="7"/>
-      <c r="D10" s="9"/>
-      <c r="E10" s="10"/>
-      <c r="F10" s="24" t="s">
-        <v>12</v>
-      </c>
-      <c r="G10" s="10"/>
-      <c r="H10" s="9"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="11"/>
-      <c r="K10" s="10"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="10"/>
-      <c r="N10" s="26" t="s">
-        <v>17</v>
-      </c>
-      <c r="O10" s="10"/>
-      <c r="P10" s="9" t="s">
-        <v>23</v>
-      </c>
-      <c r="Q10" s="10"/>
-      <c r="R10" s="5"/>
-      <c r="S10" s="10"/>
-      <c r="T10" s="12"/>
-      <c r="U10" s="14"/>
-      <c r="V10" s="13"/>
-      <c r="W10" s="14"/>
-      <c r="X10" s="15">
+      <c r="D10" s="12"/>
+      <c r="E10" s="13"/>
+      <c r="F10" s="5"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="12"/>
+      <c r="I10" s="13"/>
+      <c r="J10" s="14"/>
+      <c r="K10" s="13"/>
+      <c r="L10" s="16"/>
+      <c r="M10" s="13"/>
+      <c r="N10" s="5"/>
+      <c r="O10" s="13"/>
+      <c r="P10" s="18"/>
+      <c r="Q10" s="21"/>
+      <c r="R10" s="20"/>
+      <c r="S10" s="21"/>
+      <c r="T10" s="22">
         <v>0</v>
       </c>
-      <c r="Y10" s="14"/>
-      <c r="Z10" s="13">
+      <c r="U10" s="21"/>
+      <c r="V10" s="20">
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="2:26" ht="79.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:22" ht="79.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="B11" s="6">
         <v>3</v>
       </c>
       <c r="C11" s="7"/>
-      <c r="D11" s="9"/>
-      <c r="E11" s="10"/>
-      <c r="F11" s="24" t="s">
-        <v>13</v>
-      </c>
-      <c r="G11" s="10"/>
-      <c r="H11" s="9"/>
-      <c r="I11" s="10"/>
-      <c r="J11" s="11"/>
-      <c r="K11" s="10"/>
-      <c r="L11" s="9"/>
-      <c r="M11" s="10"/>
-      <c r="N11" s="27" t="s">
-        <v>19</v>
-      </c>
-      <c r="O11" s="10"/>
-      <c r="P11" s="9"/>
-      <c r="Q11" s="10"/>
-      <c r="R11" s="5"/>
-      <c r="S11" s="10"/>
-      <c r="T11" s="12"/>
-      <c r="U11" s="14"/>
-      <c r="V11" s="13"/>
-      <c r="W11" s="14"/>
-      <c r="X11" s="15">
+      <c r="D11" s="12"/>
+      <c r="E11" s="13"/>
+      <c r="F11" s="5"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="12"/>
+      <c r="I11" s="13"/>
+      <c r="J11" s="14"/>
+      <c r="K11" s="13"/>
+      <c r="L11" s="16"/>
+      <c r="M11" s="13"/>
+      <c r="N11" s="5"/>
+      <c r="O11" s="13"/>
+      <c r="P11" s="18"/>
+      <c r="Q11" s="21"/>
+      <c r="R11" s="20"/>
+      <c r="S11" s="21"/>
+      <c r="T11" s="22">
         <v>0</v>
       </c>
-      <c r="Y11" s="14"/>
-      <c r="Z11" s="13">
+      <c r="U11" s="21"/>
+      <c r="V11" s="20">
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="2:26" ht="79.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="P12" s="30"/>
-    </row>
-    <row r="13" spans="2:26" ht="79.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="14" spans="2:26" ht="79.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="15" spans="2:26" ht="79.5" customHeight="1" x14ac:dyDescent="0.25"/>
-    <row r="16" spans="2:26" ht="79.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="12" spans="2:22" ht="79.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="13" spans="2:22" ht="79.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="14" spans="2:22" ht="79.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="15" spans="2:22" ht="79.5" customHeight="1" x14ac:dyDescent="0.25"/>
+    <row r="16" spans="2:22" ht="79.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="17" ht="79.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="18" ht="79.5" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="19" ht="79.5" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -1777,15 +1446,18 @@
     <row r="504" ht="79.5" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="3">
+    <mergeCell ref="P6:R6"/>
     <mergeCell ref="T6:V6"/>
-    <mergeCell ref="X6:Z6"/>
-    <mergeCell ref="B2:Z4"/>
+    <mergeCell ref="B2:V4"/>
   </mergeCells>
   <conditionalFormatting sqref="B5:C8">
     <cfRule type="duplicateValues" dxfId="0" priority="2"/>
   </conditionalFormatting>
+  <hyperlinks>
+    <hyperlink ref="L9" r:id="rId1" xr:uid="{3342952E-CDC3-443D-BF48-B542992A9606}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
-  <drawing r:id="rId2"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId2"/>
+  <drawing r:id="rId3"/>
 </worksheet>
 </file>
</xml_diff>